<commit_message>
Simplificamos Grano a sus cuatro secciones principales
</commit_message>
<xml_diff>
--- a/docs/Anexo 2 - Requerimientos Grano.xlsx
+++ b/docs/Anexo 2 - Requerimientos Grano.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="4" r:id="R3f070771047d4c5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requerimiento Inicial" sheetId="3" r:id="Raada567c4c914122"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="4" r:id="R5cbf9cfd3e3e4767"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requerimiento Inicial" sheetId="3" r:id="R5671407bd55d46fa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -584,10 +584,10 @@
         <x:v>La tienda debe permitir recorrer sus páginas mediante el menú, el logo y los enlaces del pie.</x:v>
       </x:c>
       <x:c r="G2" s="16" t="str">
-        <x:v>Implementado en maqueta</x:v>
+        <x:v>Implementado en la interfaz</x:v>
       </x:c>
       <x:c r="H2" s="17" t="str">
-        <x:v>Desde cada página se puede volver al inicio y abrir catálogo, nosotros, diario, contacto, cuenta y bolsa.</x:v>
+        <x:v>Desde cada página se puede volver al inicio y abrir catálogo, nosotros y contacto; cuenta y bolsa se abren desde el pie.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="65" customHeight="1">
@@ -610,7 +610,7 @@
         <x:v>El inicio debe mostrar la identidad de Grano, una imagen principal y tres productos destacados.</x:v>
       </x:c>
       <x:c r="G3" s="16" t="str">
-        <x:v>Implementado en maqueta</x:v>
+        <x:v>Implementado en la interfaz</x:v>
       </x:c>
       <x:c r="H3" s="17" t="str">
         <x:v>Se ve el nombre Grano, una presentación, una ilustración y tres tarjetas con nombre, imagen y precio.</x:v>
@@ -636,7 +636,7 @@
         <x:v>El catálogo debe mostrar seis productos de ejemplo con imagen, nombre, precio en CLP y acceso al detalle.</x:v>
       </x:c>
       <x:c r="G4" s="16" t="str">
-        <x:v>Implementado en maqueta</x:v>
+        <x:v>Implementado en la interfaz</x:v>
       </x:c>
       <x:c r="H4" s="17" t="str">
         <x:v>Los seis productos se ven y cada enlace abre su ficha correspondiente; Añadir permanece deshabilitado.</x:v>
@@ -662,7 +662,7 @@
         <x:v>Cada producto debe tener una ficha estática con descripción, imagen y precio.</x:v>
       </x:c>
       <x:c r="G5" s="16" t="str">
-        <x:v>Implementado en maqueta</x:v>
+        <x:v>Implementado en la interfaz</x:v>
       </x:c>
       <x:c r="H5" s="17" t="str">
         <x:v>Hay seis fichas diferentes y todas permiten volver al catálogo sin agregar productos a la bolsa.</x:v>
@@ -688,10 +688,10 @@
         <x:v>La bolsa debe mostrar su estado vacío y un enlace para seguir mirando el catálogo.</x:v>
       </x:c>
       <x:c r="G6" s="16" t="str">
-        <x:v>Implementado en maqueta</x:v>
+        <x:v>Implementado en la interfaz</x:v>
       </x:c>
       <x:c r="H6" s="17" t="str">
-        <x:v>La bolsa muestra cero productos, explica que no permite comprar y tiene el botón de pago deshabilitado.</x:v>
+        <x:v>La bolsa muestra cero productos y ofrece un enlace para volver al catálogo; no procesa pagos.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="65" customHeight="1">
@@ -714,7 +714,7 @@
         <x:v>El sitio debe incluir las vistas de inicio de sesión y registro con campos etiquetados y enlaces entre ambas.</x:v>
       </x:c>
       <x:c r="G7" s="16" t="str">
-        <x:v>Implementado en maqueta</x:v>
+        <x:v>Implementado en la interfaz</x:v>
       </x:c>
       <x:c r="H7" s="17" t="str">
         <x:v>Se puede ir de ingreso a registro y volver; escribir en los campos no crea una cuenta ni inicia sesión.</x:v>
@@ -725,7 +725,7 @@
         <x:v>RF-07</x:v>
       </x:c>
       <x:c r="B8" s="16" t="str">
-        <x:v>Conocer el proyecto y el contacto</x:v>
+        <x:v>Conocer Grano y acceder al contacto</x:v>
       </x:c>
       <x:c r="C8" s="16" t="str">
         <x:v>Funcional</x:v>
@@ -737,13 +737,13 @@
         <x:v>Visitante</x:v>
       </x:c>
       <x:c r="F8" s="16" t="str">
-        <x:v>Nosotros debe presentar Grano y sus integrantes; Contacto debe mostrar nombre, correo y mensaje.</x:v>
+        <x:v>Nosotros debe presentar la identidad de Grano; Contacto debe mostrar los campos de nombre, correo y mensaje.</x:v>
       </x:c>
       <x:c r="G8" s="16" t="str">
-        <x:v>Implementado en maqueta</x:v>
+        <x:v>Implementado en la interfaz</x:v>
       </x:c>
       <x:c r="H8" s="17" t="str">
-        <x:v>Aparecen Brian Bravo y Matías Guerra; el contacto tiene etiquetas y el envío está deshabilitado.</x:v>
+        <x:v>Nosotros explica la propuesta de café y accesorios; el contacto muestra campos con etiquetas claras.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="65" customHeight="1">
@@ -751,7 +751,7 @@
         <x:v>RF-08</x:v>
       </x:c>
       <x:c r="B9" s="16" t="str">
-        <x:v>Leer el diario de Grano</x:v>
+        <x:v>Identificar las categorías del catálogo</x:v>
       </x:c>
       <x:c r="C9" s="16" t="str">
         <x:v>Funcional</x:v>
@@ -763,13 +763,13 @@
         <x:v>Visitante</x:v>
       </x:c>
       <x:c r="F9" s="16" t="str">
-        <x:v>El diario debe ofrecer dos artículos completos relacionados con café y una pieza de video.</x:v>
+        <x:v>Cada tarjeta del catálogo debe indicar si el producto es café en grano, un método o un accesorio.</x:v>
       </x:c>
       <x:c r="G9" s="16" t="str">
-        <x:v>Implementado en maqueta</x:v>
+        <x:v>Implementado en la interfaz</x:v>
       </x:c>
       <x:c r="H9" s="17" t="str">
-        <x:v>Cada tarjeta abre su artículo; ambos vuelven al diario y el artículo del ritual incluye video con controles.</x:v>
+        <x:v>Los seis productos muestran una categoría y se utilizan las etiquetas Café en grano, Métodos y Accesorios.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="65" customHeight="1">
@@ -786,13 +786,13 @@
         <x:v>Funcional de usuario</x:v>
       </x:c>
       <x:c r="E10" s="16" t="str">
-        <x:v>Visitante de la maqueta</x:v>
+        <x:v>Administrador</x:v>
       </x:c>
       <x:c r="F10" s="16" t="str">
         <x:v>El panel debe ofrecer navegación a productos, usuarios, órdenes y mensajes de ejemplo.</x:v>
       </x:c>
       <x:c r="G10" s="16" t="str">
-        <x:v>Implementado en maqueta</x:v>
+        <x:v>Implementado en la interfaz</x:v>
       </x:c>
       <x:c r="H10" s="17" t="str">
         <x:v>El enlace del pie abre el panel; su menú permite acceder a las cuatro secciones y ver una orden.</x:v>
@@ -812,13 +812,13 @@
         <x:v>Funcional de usuario</x:v>
       </x:c>
       <x:c r="E11" s="16" t="str">
-        <x:v>Visitante de la maqueta</x:v>
+        <x:v>Administrador</x:v>
       </x:c>
       <x:c r="F11" s="16" t="str">
         <x:v>Los listados deben enlazar a pantallas de creación y edición de productos y usuarios.</x:v>
       </x:c>
       <x:c r="G11" s="16" t="str">
-        <x:v>Implementado en maqueta</x:v>
+        <x:v>Implementado en la interfaz</x:v>
       </x:c>
       <x:c r="H11" s="17" t="str">
         <x:v>Se abren las cuatro pantallas, se vuelve a su listado y los botones Guardar están deshabilitados.</x:v>
@@ -873,7 +873,7 @@
         <x:v>Definido para versión 1</x:v>
       </x:c>
       <x:c r="H13" s="17" t="str">
-        <x:v>Las 26 vistas cargan la misma hoja de estilos y muestran el logo y los colores verde y crema.</x:v>
+        <x:v>Las 23 vistas cargan la misma hoja de estilos y muestran el logo y los colores verde y crema.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="65" customHeight="1">
@@ -907,7 +907,7 @@
         <x:v>RNF-04</x:v>
       </x:c>
       <x:c r="B15" s="16" t="str">
-        <x:v>Usar solo HTML CSS y Bootstrap</x:v>
+        <x:v>Compatibilidad entre navegadores</x:v>
       </x:c>
       <x:c r="C15" s="16" t="str">
         <x:v>No Funcional</x:v>
@@ -916,16 +916,16 @@
         <x:v>No funcional de producto</x:v>
       </x:c>
       <x:c r="E15" s="16" t="str">
-        <x:v>Brian Bravo y Matías Guerra</x:v>
+        <x:v>Visitante</x:v>
       </x:c>
       <x:c r="F15" s="16" t="str">
-        <x:v>La versión debe ser estática y usar únicamente HTML, CSS propio y el CSS de Bootstrap 5.3.8.</x:v>
+        <x:v>El sitio debe conservar su contenido y navegación en las versiones de escritorio de Microsoft Edge y Google Chrome.</x:v>
       </x:c>
       <x:c r="G15" s="16" t="str">
         <x:v>Definido para versión 1</x:v>
       </x:c>
       <x:c r="H15" s="17" t="str">
-        <x:v>No hay etiquetas script, manejadores JavaScript, backend, frameworks adicionales ni procesos de compilación.</x:v>
+        <x:v>Al abrir Inicio, Nuestro café, Nosotros y Contacto en ambos navegadores se ven los textos, imágenes y enlaces sin desbordamientos.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="65" customHeight="1">
@@ -959,7 +959,7 @@
         <x:v>RNF-06</x:v>
       </x:c>
       <x:c r="B17" s="17" t="str">
-        <x:v>No depender de recursos externos</x:v>
+        <x:v>Mantener disponibles los recursos visuales</x:v>
       </x:c>
       <x:c r="C17" s="17" t="str">
         <x:v>No Funcional</x:v>
@@ -971,13 +971,13 @@
         <x:v>Visitante</x:v>
       </x:c>
       <x:c r="F17" s="17" t="str">
-        <x:v>Los estilos, ilustraciones y video utilizados deben estar dentro del proyecto.</x:v>
+        <x:v>Las ilustraciones deben estar dentro del proyecto y el enlace de Bootstrap debe apuntar a una versión específica.</x:v>
       </x:c>
       <x:c r="G17" s="17" t="str">
         <x:v>Definido para versión 1</x:v>
       </x:c>
       <x:c r="H17" s="17" t="str">
-        <x:v>Al desconectar internet siguen apareciendo las imágenes y estilos y se pueden abrir todas las páginas.</x:v>
+        <x:v>Las 23 páginas cargan sus ilustraciones locales y enlazan el mismo CSS de Bootstrap 5.3.8; su carga requiere conexión a internet.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="65" customHeight="1">
@@ -1020,7 +1020,7 @@
         <x:v>No funcional de producto</x:v>
       </x:c>
       <x:c r="E19" s="17" t="str">
-        <x:v>Brian Bravo y Matías Guerra</x:v>
+        <x:v>Responsable de mantenimiento</x:v>
       </x:c>
       <x:c r="F19" s="17" t="str">
         <x:v>El CSS personalizado debe estar en un archivo externo y los componentes Bootstrap deben tener comentarios sencillos.</x:v>
@@ -1046,7 +1046,7 @@
         <x:v>No funcional de producto</x:v>
       </x:c>
       <x:c r="E20" s="17" t="str">
-        <x:v>Brian Bravo y Matías Guerra</x:v>
+        <x:v>Responsable de mantenimiento</x:v>
       </x:c>
       <x:c r="F20" s="17" t="str">
         <x:v>Todos los enlaces internos y rutas de recursos deben apuntar a archivos o secciones existentes.</x:v>
@@ -1055,7 +1055,7 @@
         <x:v>Definido para versión 1</x:v>
       </x:c>
       <x:c r="H20" s="17" t="str">
-        <x:v>La revisión de las 26 páginas no encuentra destinos internos inexistentes ni imágenes rotas.</x:v>
+        <x:v>La revisión de las 23 páginas no encuentra destinos internos inexistentes ni imágenes rotas.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="65" customHeight="1">
@@ -1063,40 +1063,40 @@
         <x:v>RNF-10</x:v>
       </x:c>
       <x:c r="B21" s="17" t="str">
-        <x:v>Registrar cambios en GitHub</x:v>
+        <x:v>Mostrar información de productos clara</x:v>
       </x:c>
       <x:c r="C21" s="17" t="str">
         <x:v>No Funcional</x:v>
       </x:c>
       <x:c r="D21" s="17" t="str">
-        <x:v>No funcional de la Organización</x:v>
+        <x:v>No funcional de producto</x:v>
       </x:c>
       <x:c r="E21" s="17" t="str">
-        <x:v>Brian Bravo y Matías Guerra</x:v>
+        <x:v>Visitante</x:v>
       </x:c>
       <x:c r="F21" s="17" t="str">
-        <x:v>Cada conjunto de cambios debe quedar registrado con un commit en español y subido al repositorio del proyecto.</x:v>
+        <x:v>Los nombres, precios y descripciones deben ser consistentes y usar términos fáciles de entender.</x:v>
       </x:c>
       <x:c r="G21" s="17" t="str">
         <x:v>Definido para versión 1</x:v>
       </x:c>
       <x:c r="H21" s="17" t="str">
-        <x:v>El historial describe tienda, administración, correcciones y documentos; la rama local queda sincronizada con GitHub.</x:v>
+        <x:v>Los seis productos conservan el mismo nombre y precio en la tarjeta y en su ficha; todos los precios se identifican como pesos chilenos.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="B24" t="str">
-        <x:v>Grano · Brian Bravo y Matías Guerra</x:v>
+        <x:v>Grano · Requisitos de la tienda</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="B25" t="str">
-        <x:v>Versión 1 · Maqueta navegable con HTML, CSS y Bootstrap</x:v>
+        <x:v>Versión 1.1 · Catálogo, navegación y atención al visitante</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="B26" t="str">
-        <x:v>Alcance: sin carrito funcional, autenticación, validaciones JavaScript ni guardado de datos.</x:v>
+        <x:v>Alcance actual: presentación de pantallas y navegación, sin procesamiento de compras o datos.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>